<commit_message>
Clientes del vendedor de Tijuana
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmacias\Desktop\RUTAS LÓGICAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC60420B-5715-4AEF-9ECE-AD3F8303DFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B49469-3C53-4501-A467-1592618A5E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{740DF47F-2FF5-45E2-939D-94824F9E772D}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">clientes!$A$1:$K$98</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="290">
   <si>
     <t>XIMENA SARAHI LOPEZ VILLASEÑOR</t>
   </si>
@@ -646,6 +646,270 @@
   </si>
   <si>
     <t>AQUILES SERDAN 575 COLONIA SANTA ANITA TLAJOMULCO DE ZUÑIGA 45645</t>
+  </si>
+  <si>
+    <t>DAVID HORACIO CABRERA BRICEÑO</t>
+  </si>
+  <si>
+    <t>BLANCA DELIA PASOS RAMOS</t>
+  </si>
+  <si>
+    <t>PINTURAS RAVI</t>
+  </si>
+  <si>
+    <t>NOELIA COTA LOPEZ</t>
+  </si>
+  <si>
+    <t>DEILY CARMINA ROJO HERNANDEZ</t>
+  </si>
+  <si>
+    <t>MANGUERAS Y SOLUCIONES INTEGRALES D PACIFICO</t>
+  </si>
+  <si>
+    <t>RANDALL ALBERTO COTA LEY</t>
+  </si>
+  <si>
+    <t>FRANCISCO CABANILLAS ORTIZ</t>
+  </si>
+  <si>
+    <t>HIRAM GERMAN NOGUERON MUNGUIA</t>
+  </si>
+  <si>
+    <t>JOSE DE LA CRUZ AMAVIZCA CHAVEZ</t>
+  </si>
+  <si>
+    <t>DESARROLLO COMERCIAL GRUJAC</t>
+  </si>
+  <si>
+    <t>YSABEL MAREZ CARDOZA</t>
+  </si>
+  <si>
+    <t>PINTURAS MARTINEZ INDA</t>
+  </si>
+  <si>
+    <t>MONICA RODRIGUEZ ALMADA</t>
+  </si>
+  <si>
+    <t>MANUEL DE JESUS MUÑOZ MENDIVIL</t>
+  </si>
+  <si>
+    <t>GASES Y EQUIPOS DE OBREGON</t>
+  </si>
+  <si>
+    <t>ANGELICA AYDEE AUDELO CRUZ</t>
+  </si>
+  <si>
+    <t>JORGE ALFONSO JACKSON CECEÑA</t>
+  </si>
+  <si>
+    <t>JUAN ALFONSO CABANILLAS FLORES</t>
+  </si>
+  <si>
+    <t>HECTOR ROJO INZUNZA</t>
+  </si>
+  <si>
+    <t>HERNAN BRASS HERNANDEZ</t>
+  </si>
+  <si>
+    <t>MARIBEL RAMIREZ MARTINEZ</t>
+  </si>
+  <si>
+    <t>CARLOS ALEJANDRO FLORES INZUNZA</t>
+  </si>
+  <si>
+    <t>IVETH ALEJANDRA PAYAN LEYVA</t>
+  </si>
+  <si>
+    <t>ANDRES VALDEZ ANGUAMEA</t>
+  </si>
+  <si>
+    <t>MATERIALES GISO</t>
+  </si>
+  <si>
+    <t>JOZHE ALONSO LOPEZ HIGUERA</t>
+  </si>
+  <si>
+    <t>ROSARIO MONCERRAT PORTILLO HERNANDEZ</t>
+  </si>
+  <si>
+    <t>PLOMERIA MODERNA</t>
+  </si>
+  <si>
+    <t>MARIA NAVA LEON</t>
+  </si>
+  <si>
+    <t>LUIS ANTONIO SPENCER</t>
+  </si>
+  <si>
+    <t>ALMA CARMINA MACHADO COTA</t>
+  </si>
+  <si>
+    <t>JUAN ENRIQUE ARMENTA SEVILLA</t>
+  </si>
+  <si>
+    <t>JAVIER ROBLES BORBOA</t>
+  </si>
+  <si>
+    <t>ARLIN SARAHI LOPEZ REYES</t>
+  </si>
+  <si>
+    <t>MARTHA LIDIA ALCANTAR MIRANDA</t>
+  </si>
+  <si>
+    <t>ORALIA GIL GALAVIZ</t>
+  </si>
+  <si>
+    <t>CHRISTIAN ABIGAIL ROJO PACHECO</t>
+  </si>
+  <si>
+    <t>CAPSA MATERIALES</t>
+  </si>
+  <si>
+    <t>OLIVIA CAMACHO SUJA</t>
+  </si>
+  <si>
+    <t>GLORIA GALAVIZ BORQUEZ</t>
+  </si>
+  <si>
+    <t>JUAN MANUEL SANCHEZ CURIEL</t>
+  </si>
+  <si>
+    <t>REYNA EVELIA AVILA VERDUGO</t>
+  </si>
+  <si>
+    <t>NYSER ARMANDO LEOPOLDO GOMEZ COTA</t>
+  </si>
+  <si>
+    <t>IVAN ANTONIO HERNANDEZ ENRIQUEZ</t>
+  </si>
+  <si>
+    <t>ALMA YOLANDA SERRANO RAMOS</t>
+  </si>
+  <si>
+    <t>BACILIO CUADRAS INZUNZA</t>
+  </si>
+  <si>
+    <t>CHRISTIAN MIGUEL LOPEZ ORTEGA</t>
+  </si>
+  <si>
+    <t>JESUS ERNESTO ORDUÑO CAMPAS</t>
+  </si>
+  <si>
+    <t>RAUL ENRIQUE LEON BOJORQUEZ</t>
+  </si>
+  <si>
+    <t>JOSE ARAMBURO LIZARRAGA</t>
+  </si>
+  <si>
+    <t>VICTOR DAVID MARTINEZ RUIZ</t>
+  </si>
+  <si>
+    <t>ALBERTO VERDUGO DELGADILLO</t>
+  </si>
+  <si>
+    <t>DIANA LORENA MORENO ROBLES</t>
+  </si>
+  <si>
+    <t>FERRETERA LA CENTRAL DE CAJEME</t>
+  </si>
+  <si>
+    <t>MANUELA DE LA CRUZ BURGOS PARRA</t>
+  </si>
+  <si>
+    <t>MARIA DE LOS ANGELES COTA VEGA</t>
+  </si>
+  <si>
+    <t>CARLOS ARMANDO ALMODOVAR MORENO</t>
+  </si>
+  <si>
+    <t>TUBOS Y MANGUERAS FLEXIBLES DEL NOR</t>
+  </si>
+  <si>
+    <t>ELSA MARIA DUARTE COZARIT</t>
+  </si>
+  <si>
+    <t>REYNALDO PADILLA BELTRAN</t>
+  </si>
+  <si>
+    <t>PAZ TORRES</t>
+  </si>
+  <si>
+    <t>FERRETERIA Y COMERCIALIZADORA DEL NOROESTE</t>
+  </si>
+  <si>
+    <t>SERGIO CARLOS VEGA FELIX</t>
+  </si>
+  <si>
+    <t>VELIA EDITH CARRILLO SUAREZ</t>
+  </si>
+  <si>
+    <t>GUADALUPE ANGULO SANTILLANES</t>
+  </si>
+  <si>
+    <t>RAMON DE JESUS FLORES CAMACHO</t>
+  </si>
+  <si>
+    <t>GUADALUPE MARTINEZ ZAMORA</t>
+  </si>
+  <si>
+    <t>PINTURAS DE CAJEME</t>
+  </si>
+  <si>
+    <t>TANIA IVONNE MANCILLAS VALDEZ</t>
+  </si>
+  <si>
+    <t>EQUIPOS Y PARTES GLOBAL</t>
+  </si>
+  <si>
+    <t>PINTURAS ESPECIALES DE LOS MOCHIS</t>
+  </si>
+  <si>
+    <t>LAURA LYDIA MUY FLORES</t>
+  </si>
+  <si>
+    <t>FRANCISCO G RAMIREZ</t>
+  </si>
+  <si>
+    <t>SERGIO HUMBERTO RUBIO LOPEZ</t>
+  </si>
+  <si>
+    <t>JOHANA IVETTE VAZQUEZ MEDINA</t>
+  </si>
+  <si>
+    <t>YANKY AUTO SHOP</t>
+  </si>
+  <si>
+    <t>MANUEL TRINIDAD CHIN DUARTE</t>
+  </si>
+  <si>
+    <t>CARLOS ARMANDO CUADRAS CANO</t>
+  </si>
+  <si>
+    <t>JESUS MANUEL MARTINEZ LUGO</t>
+  </si>
+  <si>
+    <t>GILBERTO ENRIQUE GASTELUM ESPINOZA</t>
+  </si>
+  <si>
+    <t>KARLA GARNICA MELLOY</t>
+  </si>
+  <si>
+    <t>CARLOS MENDOZA LUNA</t>
+  </si>
+  <si>
+    <t>LOGISTICA ZARR</t>
+  </si>
+  <si>
+    <t>ROBERTO HINOJOSA NIEBLAS</t>
+  </si>
+  <si>
+    <t>MATILDE INZUNZA GUILLEN</t>
+  </si>
+  <si>
+    <t>ANAHY CAZAREZ ARMENTA</t>
+  </si>
+  <si>
+    <t>YASBEL GUADALUPE OCHOA DIAZ</t>
   </si>
 </sst>
 </file>
@@ -716,7 +980,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -731,12 +995,35 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1066,11 +1353,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1E63F05-B3C2-4FFE-ACBF-95CFEEB9BDFD}">
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K186"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.26953125" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.54296875" style="6" bestFit="1" customWidth="1"/>
@@ -4304,8 +4591,979 @@
         <v>190</v>
       </c>
     </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>50000416</v>
+      </c>
+      <c r="B99" s="12">
+        <v>621795</v>
+      </c>
+      <c r="C99" s="13" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>50000416</v>
+      </c>
+      <c r="B100" s="12">
+        <v>621251</v>
+      </c>
+      <c r="C100" s="13" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>50000416</v>
+      </c>
+      <c r="B101" s="12">
+        <v>1046</v>
+      </c>
+      <c r="C101" s="13" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>50000416</v>
+      </c>
+      <c r="B102" s="12">
+        <v>621641</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>50000416</v>
+      </c>
+      <c r="B103" s="12">
+        <v>233979</v>
+      </c>
+      <c r="C103" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <v>50000416</v>
+      </c>
+      <c r="B104" s="12">
+        <v>235061</v>
+      </c>
+      <c r="C104" s="14" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <v>50000416</v>
+      </c>
+      <c r="B105" s="12">
+        <v>621509</v>
+      </c>
+      <c r="C105" s="13" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <v>50000416</v>
+      </c>
+      <c r="B106" s="12">
+        <v>620295</v>
+      </c>
+      <c r="C106" s="13" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <v>50000416</v>
+      </c>
+      <c r="B107" s="12">
+        <v>621886</v>
+      </c>
+      <c r="C107" s="13" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <v>50000416</v>
+      </c>
+      <c r="B108" s="12">
+        <v>621242</v>
+      </c>
+      <c r="C108" s="14" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <v>50000416</v>
+      </c>
+      <c r="B109" s="12">
+        <v>621780</v>
+      </c>
+      <c r="C109" s="14" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <v>50000416</v>
+      </c>
+      <c r="B110" s="12">
+        <v>620850</v>
+      </c>
+      <c r="C110" s="14" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <v>50000416</v>
+      </c>
+      <c r="B111" s="12">
+        <v>1508</v>
+      </c>
+      <c r="C111" s="14" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <v>50000416</v>
+      </c>
+      <c r="B112" s="12">
+        <v>234183</v>
+      </c>
+      <c r="C112" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>50000416</v>
+      </c>
+      <c r="B113" s="12">
+        <v>347182</v>
+      </c>
+      <c r="C113" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>50000416</v>
+      </c>
+      <c r="B114" s="12">
+        <v>621897</v>
+      </c>
+      <c r="C114" s="14" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>50000416</v>
+      </c>
+      <c r="B115" s="12">
+        <v>1000264</v>
+      </c>
+      <c r="C115" s="13" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>50000416</v>
+      </c>
+      <c r="B116" s="12">
+        <v>621608</v>
+      </c>
+      <c r="C116" s="13" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>50000416</v>
+      </c>
+      <c r="B117" s="12">
+        <v>621781</v>
+      </c>
+      <c r="C117" s="14" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>50000416</v>
+      </c>
+      <c r="B118" s="12">
+        <v>621845</v>
+      </c>
+      <c r="C118" s="14" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>50000416</v>
+      </c>
+      <c r="B119" s="12">
+        <v>621887</v>
+      </c>
+      <c r="C119" s="13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>50000416</v>
+      </c>
+      <c r="B120" s="12">
+        <v>621316</v>
+      </c>
+      <c r="C120" s="14" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121">
+        <v>50000416</v>
+      </c>
+      <c r="B121" s="12">
+        <v>620445</v>
+      </c>
+      <c r="C121" s="14" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122">
+        <v>50000416</v>
+      </c>
+      <c r="B122" s="12">
+        <v>621596</v>
+      </c>
+      <c r="C122" s="14" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A123">
+        <v>50000416</v>
+      </c>
+      <c r="B123" s="12">
+        <v>340708</v>
+      </c>
+      <c r="C123" s="13" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A124">
+        <v>50000416</v>
+      </c>
+      <c r="B124" s="12">
+        <v>234382</v>
+      </c>
+      <c r="C124" s="13" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125">
+        <v>50000416</v>
+      </c>
+      <c r="B125" s="12">
+        <v>341184</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126">
+        <v>50000416</v>
+      </c>
+      <c r="B126" s="12">
+        <v>343306</v>
+      </c>
+      <c r="C126" s="13" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127">
+        <v>50000416</v>
+      </c>
+      <c r="B127" s="12">
+        <v>621846</v>
+      </c>
+      <c r="C127" s="13" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>50000416</v>
+      </c>
+      <c r="B128" s="12">
+        <v>620782</v>
+      </c>
+      <c r="C128" s="14" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>50000416</v>
+      </c>
+      <c r="B129" s="12">
+        <v>621578</v>
+      </c>
+      <c r="C129" s="14" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>50000416</v>
+      </c>
+      <c r="B130" s="12">
+        <v>621404</v>
+      </c>
+      <c r="C130" s="14" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131">
+        <v>50000416</v>
+      </c>
+      <c r="B131" s="12">
+        <v>346207</v>
+      </c>
+      <c r="C131" s="13" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132">
+        <v>50000416</v>
+      </c>
+      <c r="B132" s="12">
+        <v>620292</v>
+      </c>
+      <c r="C132" s="13" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133">
+        <v>50000416</v>
+      </c>
+      <c r="B133" s="12">
+        <v>621840</v>
+      </c>
+      <c r="C133" s="14" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134">
+        <v>50000416</v>
+      </c>
+      <c r="B134" s="12">
+        <v>621459</v>
+      </c>
+      <c r="C134" s="14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135">
+        <v>50000416</v>
+      </c>
+      <c r="B135" s="12">
+        <v>235022</v>
+      </c>
+      <c r="C135" s="14" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A136">
+        <v>50000416</v>
+      </c>
+      <c r="B136" s="12">
+        <v>234255</v>
+      </c>
+      <c r="C136" s="13" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A137">
+        <v>50000416</v>
+      </c>
+      <c r="B137" s="12">
+        <v>621525</v>
+      </c>
+      <c r="C137" s="14" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A138">
+        <v>50000416</v>
+      </c>
+      <c r="B138" s="12">
+        <v>234840</v>
+      </c>
+      <c r="C138" s="14" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A139">
+        <v>50000416</v>
+      </c>
+      <c r="B139" s="12">
+        <v>235121</v>
+      </c>
+      <c r="C139" s="14" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A140">
+        <v>50000416</v>
+      </c>
+      <c r="B140" s="12">
+        <v>345366</v>
+      </c>
+      <c r="C140" s="14" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A141">
+        <v>50000416</v>
+      </c>
+      <c r="B141" s="12">
+        <v>234841</v>
+      </c>
+      <c r="C141" s="14" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A142">
+        <v>50000416</v>
+      </c>
+      <c r="B142" s="12">
+        <v>234791</v>
+      </c>
+      <c r="C142" s="14" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A143">
+        <v>50000416</v>
+      </c>
+      <c r="B143" s="12">
+        <v>234634</v>
+      </c>
+      <c r="C143" s="14" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A144">
+        <v>50000416</v>
+      </c>
+      <c r="B144" s="12">
+        <v>621799</v>
+      </c>
+      <c r="C144" s="14" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A145">
+        <v>50000416</v>
+      </c>
+      <c r="B145" s="12">
+        <v>342130</v>
+      </c>
+      <c r="C145" s="14" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A146">
+        <v>50000416</v>
+      </c>
+      <c r="B146" s="12">
+        <v>621787</v>
+      </c>
+      <c r="C146" s="14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A147">
+        <v>50000416</v>
+      </c>
+      <c r="B147" s="12">
+        <v>621607</v>
+      </c>
+      <c r="C147" s="14" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A148">
+        <v>50000416</v>
+      </c>
+      <c r="B148" s="12">
+        <v>621675</v>
+      </c>
+      <c r="C148" s="14" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A149">
+        <v>50000416</v>
+      </c>
+      <c r="B149" s="12">
+        <v>621320</v>
+      </c>
+      <c r="C149" s="13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A150">
+        <v>50000416</v>
+      </c>
+      <c r="B150" s="12">
+        <v>621900</v>
+      </c>
+      <c r="C150" s="13" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A151">
+        <v>50000416</v>
+      </c>
+      <c r="B151" s="12">
+        <v>1000263</v>
+      </c>
+      <c r="C151" s="14" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A152">
+        <v>50000416</v>
+      </c>
+      <c r="B152" s="12">
+        <v>346213</v>
+      </c>
+      <c r="C152" s="13" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A153">
+        <v>50000416</v>
+      </c>
+      <c r="B153" s="12">
+        <v>620567</v>
+      </c>
+      <c r="C153" s="14" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A154">
+        <v>50000416</v>
+      </c>
+      <c r="B154" s="12">
+        <v>621885</v>
+      </c>
+      <c r="C154" s="14" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A155">
+        <v>50000416</v>
+      </c>
+      <c r="B155" s="12">
+        <v>348080</v>
+      </c>
+      <c r="C155" s="14" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A156">
+        <v>50000416</v>
+      </c>
+      <c r="B156" s="12">
+        <v>621802</v>
+      </c>
+      <c r="C156" s="14" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A157">
+        <v>50000416</v>
+      </c>
+      <c r="B157" s="12">
+        <v>621834</v>
+      </c>
+      <c r="C157" s="14" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A158">
+        <v>50000416</v>
+      </c>
+      <c r="B158" s="12">
+        <v>621817</v>
+      </c>
+      <c r="C158" s="14" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A159">
+        <v>50000416</v>
+      </c>
+      <c r="B159" s="12">
+        <v>621796</v>
+      </c>
+      <c r="C159" s="14" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A160">
+        <v>50000416</v>
+      </c>
+      <c r="B160" s="12">
+        <v>621790</v>
+      </c>
+      <c r="C160" s="14" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A161">
+        <v>50000416</v>
+      </c>
+      <c r="B161" s="12">
+        <v>621903</v>
+      </c>
+      <c r="C161" s="13" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A162">
+        <v>50000416</v>
+      </c>
+      <c r="B162" s="12">
+        <v>621677</v>
+      </c>
+      <c r="C162" s="13" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A163">
+        <v>50000416</v>
+      </c>
+      <c r="B163" s="12">
+        <v>340315</v>
+      </c>
+      <c r="C163" s="14" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A164">
+        <v>50000416</v>
+      </c>
+      <c r="B164" s="12">
+        <v>172861</v>
+      </c>
+      <c r="C164" s="13" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A165">
+        <v>50000416</v>
+      </c>
+      <c r="B165" s="12">
+        <v>620935</v>
+      </c>
+      <c r="C165" s="13" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A166">
+        <v>50000416</v>
+      </c>
+      <c r="B166" s="12">
+        <v>347296</v>
+      </c>
+      <c r="C166" s="14" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A167">
+        <v>50000416</v>
+      </c>
+      <c r="B167" s="12">
+        <v>620942</v>
+      </c>
+      <c r="C167" s="14" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A168">
+        <v>50000416</v>
+      </c>
+      <c r="B168" s="12">
+        <v>621481</v>
+      </c>
+      <c r="C168" s="14" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A169">
+        <v>50000416</v>
+      </c>
+      <c r="B169" s="12">
+        <v>620834</v>
+      </c>
+      <c r="C169" s="14" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A170">
+        <v>50000416</v>
+      </c>
+      <c r="B170" s="12">
+        <v>620180</v>
+      </c>
+      <c r="C170" s="14" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A171">
+        <v>50000416</v>
+      </c>
+      <c r="B171" s="12">
+        <v>621601</v>
+      </c>
+      <c r="C171" s="13" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A172">
+        <v>50000416</v>
+      </c>
+      <c r="B172" s="12">
+        <v>620884</v>
+      </c>
+      <c r="C172" s="14" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A173">
+        <v>50000416</v>
+      </c>
+      <c r="B173" s="12">
+        <v>621454</v>
+      </c>
+      <c r="C173" s="14" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A174">
+        <v>50000416</v>
+      </c>
+      <c r="B174" s="12">
+        <v>621905</v>
+      </c>
+      <c r="C174" s="13" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A175">
+        <v>50000416</v>
+      </c>
+      <c r="B175" s="12">
+        <v>621804</v>
+      </c>
+      <c r="C175" s="14" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A176">
+        <v>50000416</v>
+      </c>
+      <c r="B176" s="12">
+        <v>347056</v>
+      </c>
+      <c r="C176" s="14" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A177">
+        <v>50000416</v>
+      </c>
+      <c r="B177" s="12">
+        <v>234177</v>
+      </c>
+      <c r="C177" s="13" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A178">
+        <v>50000416</v>
+      </c>
+      <c r="B178" s="12">
+        <v>621308</v>
+      </c>
+      <c r="C178" s="14" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A179">
+        <v>50000416</v>
+      </c>
+      <c r="B179" s="12">
+        <v>1001122</v>
+      </c>
+      <c r="C179" s="13" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A180">
+        <v>50000416</v>
+      </c>
+      <c r="B180" s="12">
+        <v>1001126</v>
+      </c>
+      <c r="C180" s="13" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A181">
+        <v>50000416</v>
+      </c>
+      <c r="B181" s="12">
+        <v>1001004</v>
+      </c>
+      <c r="C181" s="14" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A182">
+        <v>50000416</v>
+      </c>
+      <c r="B182" s="12">
+        <v>346002</v>
+      </c>
+      <c r="C182" s="13" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A183">
+        <v>50000416</v>
+      </c>
+      <c r="B183" s="15">
+        <v>1001854</v>
+      </c>
+      <c r="C183" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A184">
+        <v>50000416</v>
+      </c>
+      <c r="B184" s="15">
+        <v>1002307</v>
+      </c>
+      <c r="C184" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A185">
+        <v>50000416</v>
+      </c>
+      <c r="B185" s="15">
+        <v>1002361</v>
+      </c>
+      <c r="C185" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A186">
+        <v>50000416</v>
+      </c>
+      <c r="B186" s="15">
+        <v>621888</v>
+      </c>
+      <c r="C186" t="s">
+        <v>289</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K98" xr:uid="{F1E63F05-B3C2-4FFE-ACBF-95CFEEB9BDFD}"/>
+  <conditionalFormatting sqref="B99:B186">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>